<commit_message>
Corrige MAPA-ORG v1.1 — substitui titulares na Seção 5 / aba Titular x Evidência pela equipe da proposta de entrevistas
Reverte a alteração indevida de RACI da versão anterior e aplica apenas a
substituição de titulares na Seção 5 (docx) / aba Titular x Evidência (xlsx),
conforme a proposta de papéis para entrevistas MPS-SW Nível C (equipe
principal + apoio opcional). Coluna de evidência mantida intacta; RACI,
competências e rastreabilidade sem alteração.

https://claude.ai/code/session_016t8bKHqvLbMdZ5bLTCngAs
</commit_message>
<xml_diff>
--- a/MAPA-ORG-002_Papeis-e-Responsabilidades_TIMEWARE_v1.1.xlsx
+++ b/MAPA-ORG-002_Papeis-e-Responsabilidades_TIMEWARE_v1.1.xlsx
@@ -807,7 +807,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Atualização da distribuição de responsáveis por processo (RACI) conforme proposta de papéis para entrevistas MPS-SW Nível C</t>
+          <t>Atualização dos titulares na Seção 5 (Papel × Titular × Evidência) para a equipe da proposta de papéis para entrevistas MPS-SW Nível C (equipe principal + apoio opcional); coluna de evidência mantida.</t>
         </is>
       </c>
     </row>
@@ -881,17 +881,17 @@
       </c>
       <c r="B4" s="18" t="inlineStr">
         <is>
+          <t>Time de Melhoria Contínua</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
           <t>Gerente de Projeto</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
-        <is>
-          <t>Gerente de Projeto</t>
-        </is>
-      </c>
       <c r="D4" s="18" t="inlineStr">
         <is>
-          <t>SEPG (C); COO (I)</t>
+          <t>GQA (C); COO (I)</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="B5" s="19" t="inlineStr">
         <is>
-          <t>Gerente de Projeto / PO</t>
+          <t>Time de Melhoria Contínua</t>
         </is>
       </c>
       <c r="C5" s="19" t="inlineStr">
@@ -913,7 +913,7 @@
       </c>
       <c r="D5" s="19" t="inlineStr">
         <is>
-          <t>SEPG (C); Cliente (C)</t>
+          <t>GQA (C); Cliente (C)</t>
         </is>
       </c>
     </row>
@@ -925,7 +925,7 @@
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>Tech Lead</t>
+          <t>Time de Melhoria Contínua</t>
         </is>
       </c>
       <c r="C6" s="18" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>Tech Lead</t>
+          <t>Time de Melhoria Contínua</t>
         </is>
       </c>
       <c r="C7" s="19" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="B8" s="18" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>Time de Melhoria Contínua</t>
         </is>
       </c>
       <c r="C8" s="18" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="D8" s="18" t="inlineStr">
         <is>
-          <t>Gerente de Projeto (C); Cliente (C)</t>
+          <t>GQA (C); Cliente (C)</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>Tech Lead</t>
+          <t>Time de Melhoria Contínua</t>
         </is>
       </c>
       <c r="C9" s="19" t="inlineStr">
@@ -1001,7 +1001,7 @@
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>GQA (C); DevOps (C)</t>
+          <t>GQA (C)</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1013,7 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>Time de Melhoria Contínua / SEPG</t>
+          <t>COO</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="D10" s="18" t="inlineStr">
         <is>
-          <t>RH / Capacitação (C); Sponsor / Portfólio (I)</t>
+          <t>COO (A)</t>
         </is>
       </c>
     </row>
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>Time de Melhoria Contínua / SEPG</t>
+          <t>Time de Melhoria Contínua</t>
         </is>
       </c>
       <c r="C11" s="19" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>Gerente de Projeto (C); COO (I)</t>
+          <t>COO (I)</t>
         </is>
       </c>
     </row>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="D12" s="18" t="inlineStr">
         <is>
-          <t>RH / Capacitação (C); Sponsor / Portfólio (I)</t>
+          <t>COO (A)</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="B13" s="19" t="inlineStr">
         <is>
-          <t>Tech Lead</t>
+          <t>Time de Melhoria Contínua</t>
         </is>
       </c>
       <c r="C13" s="19" t="inlineStr">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>SEPG (C) em decisões organizacionais; GQA (C)</t>
+          <t>COO (C); GQA (C)</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="B14" s="18" t="inlineStr">
         <is>
-          <t>Time de Melhoria Contínua / SEPG</t>
+          <t>COO</t>
         </is>
       </c>
       <c r="C14" s="18" t="inlineStr">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="D14" s="18" t="inlineStr">
         <is>
-          <t>CEO (C); Sponsor / Portfólio (C)</t>
+          <t>GQA (C); COO (A)</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1123,7 @@
       </c>
       <c r="B15" s="19" t="inlineStr">
         <is>
-          <t>Time de Melhoria Contínua / SEPG</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>CEO (C); Sponsor / Portfólio (C)</t>
+          <t>CEO (A)</t>
         </is>
       </c>
     </row>
@@ -3456,7 +3456,7 @@
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>Renan Kioshi, Raony Chagas, Fernando Oliveira, Henry Komatsu</t>
+          <t>Renan Kioshi, Raony Chagas</t>
         </is>
       </c>
       <c r="C6" s="18" t="inlineStr">
@@ -3473,7 +3473,7 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>Caroline Jenifer (Carol), Jonatan Silva, Letícia Moraes</t>
+          <t>Caroline Jenifer (Carol)</t>
         </is>
       </c>
       <c r="C7" s="19" t="inlineStr">
@@ -3490,7 +3490,7 @@
       </c>
       <c r="B8" s="18" t="inlineStr">
         <is>
-          <t>Rafael Cunha</t>
+          <t>Flávio Fernandes</t>
         </is>
       </c>
       <c r="C8" s="18" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>Mariana Teixeira</t>
+          <t>Cézar (Velázquez)</t>
         </is>
       </c>
       <c r="C9" s="19" t="inlineStr">
@@ -3524,7 +3524,7 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>Flávio Fernandes</t>
+          <t>Silvio Baroni</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
@@ -3541,7 +3541,7 @@
       </c>
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>Patricia Lima, Silvio Baroni (coord.), Mariana Teixeira</t>
+          <t>Silvio Baroni</t>
         </is>
       </c>
       <c r="C11" s="19" t="inlineStr">
@@ -3575,7 +3575,7 @@
       </c>
       <c r="B13" s="19" t="inlineStr">
         <is>
-          <t>Thiago Nunes</t>
+          <t>Silvio Baroni</t>
         </is>
       </c>
       <c r="C13" s="19" t="inlineStr">
@@ -3592,7 +3592,7 @@
       </c>
       <c r="B14" s="18" t="inlineStr">
         <is>
-          <t>Guilherme Gomes, Camila Ferreira</t>
+          <t>Guilherme Gomes</t>
         </is>
       </c>
       <c r="C14" s="18" t="inlineStr">
@@ -3626,7 +3626,7 @@
       </c>
       <c r="B16" s="18" t="inlineStr">
         <is>
-          <t>COO (Operações)</t>
+          <t>Wilson Yamada</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">

</xml_diff>